<commit_message>
refactor: upgrade ranking engine to TOPSIS & add interactive counterfactual simulator
- Implemented mathematically principled TOPSIS multi-criteria decision ranker.
- Added interactive Counterfactual Simulation & Skill Gaps tab to Candidate Details.
- Regenerated CSV and XLSX submissions using calibrated TOPSIS closeness metrics.
- Aligned fix_and_rerank pipeline execution script with production ranking core.
</commit_message>
<xml_diff>
--- a/data/submission.xlsx
+++ b/data/submission.xlsx
@@ -465,7 +465,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8322000000000001</v>
+        <v>0.961599</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -481,14 +481,14 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>cand_0737</t>
+          <t>cand_0936</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>0.821837</v>
+        <v>0.946058</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -504,14 +504,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>cand_0419</t>
+          <t>cand_0844</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>0.820106</v>
+        <v>0.940347</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -527,14 +527,14 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>cand_0844</t>
+          <t>cand_0419</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>0.818634</v>
+        <v>0.938563</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -550,14 +550,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>cand_0202</t>
+          <t>cand_0156</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>0.81696</v>
+        <v>0.938281</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -573,14 +573,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>cand_0936</t>
+          <t>cand_0091</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8133359999999999</v>
+        <v>0.936964</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -596,14 +596,14 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cand_0156</t>
+          <t>cand_0202</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>0.811392</v>
+        <v>0.936826</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -619,14 +619,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cand_0062</t>
+          <t>cand_0332</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>0.810551</v>
+        <v>0.936738</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -642,14 +642,14 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>cand_0091</t>
+          <t>cand_0737</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>0.8098</v>
+        <v>0.933917</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -665,14 +665,14 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>cand_0332</t>
+          <t>cand_0127</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>0.809033</v>
+        <v>0.927675</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -688,14 +688,14 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>cand_0956</t>
+          <t>cand_0722</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>0.805464</v>
+        <v>0.92675</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -711,14 +711,14 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>cand_0872</t>
+          <t>cand_0062</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>0.805124</v>
+        <v>0.926669</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -734,14 +734,14 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>cand_0337</t>
+          <t>cand_0592</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>0.8041509999999999</v>
+        <v>0.9265679999999999</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -764,7 +764,7 @@
         <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>0.803361</v>
+        <v>0.924072</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -787,7 +787,7 @@
         <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>0.801581</v>
+        <v>0.923084</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -803,14 +803,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>cand_0592</t>
+          <t>cand_0638</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" t="n">
-        <v>0.798594</v>
+        <v>0.921457</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -826,14 +826,14 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>cand_0722</t>
+          <t>cand_0337</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>0.793888</v>
+        <v>0.918802</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -849,14 +849,14 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cand_0127</t>
+          <t>cand_0185</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>18</v>
       </c>
       <c r="C19" t="n">
-        <v>0.791791</v>
+        <v>0.91777</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -872,14 +872,14 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>cand_0638</t>
+          <t>cand_0088</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>19</v>
       </c>
       <c r="C20" t="n">
-        <v>0.790736</v>
+        <v>0.915041</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -895,14 +895,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>cand_0826</t>
+          <t>cand_0272</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>0.790666</v>
+        <v>0.914465</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -918,14 +918,14 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>cand_0246</t>
+          <t>cand_0956</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>21</v>
       </c>
       <c r="C22" t="n">
-        <v>0.790498</v>
+        <v>0.9143559999999999</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -941,14 +941,14 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>cand_0111</t>
+          <t>cand_0170</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>0.788454</v>
+        <v>0.912558</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -964,14 +964,14 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>cand_0494</t>
+          <t>cand_0872</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>23</v>
       </c>
       <c r="C24" t="n">
-        <v>0.787709</v>
+        <v>0.912301</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -994,7 +994,7 @@
         <v>24</v>
       </c>
       <c r="C25" t="n">
-        <v>0.785488</v>
+        <v>0.911064</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1010,14 +1010,14 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>cand_0809</t>
+          <t>cand_0886</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>25</v>
       </c>
       <c r="C26" t="n">
-        <v>0.785366</v>
+        <v>0.909658</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1033,14 +1033,14 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>cand_0185</t>
+          <t>cand_0111</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>26</v>
       </c>
       <c r="C27" t="n">
-        <v>0.782711</v>
+        <v>0.909586</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1056,14 +1056,14 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>cand_0021</t>
+          <t>cand_0647</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>27</v>
       </c>
       <c r="C28" t="n">
-        <v>0.782477</v>
+        <v>0.9091</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1079,14 +1079,14 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>cand_0647</t>
+          <t>cand_0269</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>28</v>
       </c>
       <c r="C29" t="n">
-        <v>0.781284</v>
+        <v>0.908754</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1102,14 +1102,14 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>cand_0272</t>
+          <t>cand_0494</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>29</v>
       </c>
       <c r="C30" t="n">
-        <v>0.780437</v>
+        <v>0.908477</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1125,14 +1125,14 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>cand_0170</t>
+          <t>cand_0826</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>30</v>
       </c>
       <c r="C31" t="n">
-        <v>0.779563</v>
+        <v>0.906522</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1148,14 +1148,14 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>cand_0856</t>
+          <t>cand_0021</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>31</v>
       </c>
       <c r="C32" t="n">
-        <v>0.779453</v>
+        <v>0.906416</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1171,14 +1171,14 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>cand_0886</t>
+          <t>cand_0246</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>32</v>
       </c>
       <c r="C33" t="n">
-        <v>0.779108</v>
+        <v>0.905596</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1194,14 +1194,14 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>cand_0088</t>
+          <t>cand_0505</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>33</v>
       </c>
       <c r="C34" t="n">
-        <v>0.778859</v>
+        <v>0.904908</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1224,7 +1224,7 @@
         <v>34</v>
       </c>
       <c r="C35" t="n">
-        <v>0.77801</v>
+        <v>0.903547</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1240,14 +1240,14 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>cand_0602</t>
+          <t>cand_0529</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>35</v>
       </c>
       <c r="C36" t="n">
-        <v>0.777248</v>
+        <v>0.902655</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1263,14 +1263,14 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>cand_0269</t>
+          <t>cand_0122</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>36</v>
       </c>
       <c r="C37" t="n">
-        <v>0.775478</v>
+        <v>0.90126</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1286,14 +1286,14 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>cand_0501</t>
+          <t>cand_0809</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>37</v>
       </c>
       <c r="C38" t="n">
-        <v>0.774174</v>
+        <v>0.899346</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1316,7 +1316,7 @@
         <v>38</v>
       </c>
       <c r="C39" t="n">
-        <v>0.773134</v>
+        <v>0.898749</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1332,14 +1332,14 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>cand_0684</t>
+          <t>cand_0508</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>39</v>
       </c>
       <c r="C40" t="n">
-        <v>0.773104</v>
+        <v>0.898235</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1355,14 +1355,14 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>cand_0433</t>
+          <t>cand_0501</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>40</v>
       </c>
       <c r="C41" t="n">
-        <v>0.772425</v>
+        <v>0.8973</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1378,14 +1378,14 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>cand_0097</t>
+          <t>cand_0618</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>41</v>
       </c>
       <c r="C42" t="n">
-        <v>0.772203</v>
+        <v>0.897115</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1401,14 +1401,14 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>cand_0505</t>
+          <t>cand_0998</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>42</v>
       </c>
       <c r="C43" t="n">
-        <v>0.77169</v>
+        <v>0.8969200000000001</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1431,7 +1431,7 @@
         <v>43</v>
       </c>
       <c r="C44" t="n">
-        <v>0.769884</v>
+        <v>0.896045</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1447,14 +1447,14 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>cand_0773</t>
+          <t>cand_0856</t>
         </is>
       </c>
       <c r="B45" t="n">
         <v>44</v>
       </c>
       <c r="C45" t="n">
-        <v>0.768807</v>
+        <v>0.895321</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1470,14 +1470,14 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>cand_0772</t>
+          <t>cand_0427</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>45</v>
       </c>
       <c r="C46" t="n">
-        <v>0.767539</v>
+        <v>0.894045</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1493,14 +1493,14 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>cand_0122</t>
+          <t>cand_0772</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>46</v>
       </c>
       <c r="C47" t="n">
-        <v>0.766936</v>
+        <v>0.891879</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1516,14 +1516,14 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>cand_0831</t>
+          <t>cand_0203</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>47</v>
       </c>
       <c r="C48" t="n">
-        <v>0.766811</v>
+        <v>0.890361</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1539,14 +1539,14 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>cand_0588</t>
+          <t>cand_0221</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>48</v>
       </c>
       <c r="C49" t="n">
-        <v>0.766051</v>
+        <v>0.889374</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1562,14 +1562,14 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>cand_0508</t>
+          <t>cand_0831</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>49</v>
       </c>
       <c r="C50" t="n">
-        <v>0.765674</v>
+        <v>0.888646</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1585,14 +1585,14 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>cand_0618</t>
+          <t>cand_0079</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>50</v>
       </c>
       <c r="C51" t="n">
-        <v>0.765437</v>
+        <v>0.888616</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -1608,14 +1608,14 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>cand_0483</t>
+          <t>cand_0470</t>
         </is>
       </c>
       <c r="B52" t="n">
         <v>51</v>
       </c>
       <c r="C52" t="n">
-        <v>0.7646849999999999</v>
+        <v>0.888313</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
@@ -1631,14 +1631,14 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>cand_0221</t>
+          <t>cand_0163</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>52</v>
       </c>
       <c r="C53" t="n">
-        <v>0.763019</v>
+        <v>0.886999</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
@@ -1654,14 +1654,14 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>cand_0363</t>
+          <t>cand_0433</t>
         </is>
       </c>
       <c r="B54" t="n">
         <v>53</v>
       </c>
       <c r="C54" t="n">
-        <v>0.762849</v>
+        <v>0.886518</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -1677,14 +1677,14 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>cand_0529</t>
+          <t>cand_0372</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>54</v>
       </c>
       <c r="C55" t="n">
-        <v>0.762066</v>
+        <v>0.885612</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
@@ -1700,14 +1700,14 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>cand_0998</t>
+          <t>cand_0063</t>
         </is>
       </c>
       <c r="B56" t="n">
         <v>55</v>
       </c>
       <c r="C56" t="n">
-        <v>0.759621</v>
+        <v>0.885588</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
@@ -1723,14 +1723,14 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>cand_0653</t>
+          <t>cand_0773</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>56</v>
       </c>
       <c r="C57" t="n">
-        <v>0.7574920000000001</v>
+        <v>0.885136</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -1746,14 +1746,14 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>cand_0623</t>
+          <t>cand_0837</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>57</v>
       </c>
       <c r="C58" t="n">
-        <v>0.755814</v>
+        <v>0.884973</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -1769,14 +1769,14 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>cand_0079</t>
+          <t>cand_0653</t>
         </is>
       </c>
       <c r="B59" t="n">
         <v>58</v>
       </c>
       <c r="C59" t="n">
-        <v>0.755497</v>
+        <v>0.882467</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
@@ -1792,14 +1792,14 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>cand_0063</t>
+          <t>cand_0965</t>
         </is>
       </c>
       <c r="B60" t="n">
         <v>59</v>
       </c>
       <c r="C60" t="n">
-        <v>0.755154</v>
+        <v>0.882307</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
@@ -1815,14 +1815,14 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>cand_0965</t>
+          <t>cand_0483</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>60</v>
       </c>
       <c r="C61" t="n">
-        <v>0.752283</v>
+        <v>0.881575</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -1838,14 +1838,14 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>cand_0427</t>
+          <t>cand_0090</t>
         </is>
       </c>
       <c r="B62" t="n">
         <v>61</v>
       </c>
       <c r="C62" t="n">
-        <v>0.752277</v>
+        <v>0.881121</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
@@ -1861,14 +1861,14 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>cand_0418</t>
+          <t>cand_0363</t>
         </is>
       </c>
       <c r="B63" t="n">
         <v>62</v>
       </c>
       <c r="C63" t="n">
-        <v>0.75174</v>
+        <v>0.8806890000000001</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
@@ -1884,14 +1884,14 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>cand_0739</t>
+          <t>cand_0253</t>
         </is>
       </c>
       <c r="B64" t="n">
         <v>63</v>
       </c>
       <c r="C64" t="n">
-        <v>0.750561</v>
+        <v>0.878386</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
@@ -1907,14 +1907,14 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>cand_0440</t>
+          <t>cand_0766</t>
         </is>
       </c>
       <c r="B65" t="n">
         <v>64</v>
       </c>
       <c r="C65" t="n">
-        <v>0.7483649999999999</v>
+        <v>0.878365</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
@@ -1930,14 +1930,14 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>cand_0926</t>
+          <t>cand_0160</t>
         </is>
       </c>
       <c r="B66" t="n">
         <v>65</v>
       </c>
       <c r="C66" t="n">
-        <v>0.747819</v>
+        <v>0.878045</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -1953,14 +1953,14 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>cand_0140</t>
+          <t>cand_0082</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>66</v>
       </c>
       <c r="C67" t="n">
-        <v>0.746856</v>
+        <v>0.876559</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -1976,14 +1976,14 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>cand_0253</t>
+          <t>cand_0588</t>
         </is>
       </c>
       <c r="B68" t="n">
         <v>67</v>
       </c>
       <c r="C68" t="n">
-        <v>0.746451</v>
+        <v>0.875894</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -1999,14 +1999,14 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>cand_0163</t>
+          <t>cand_0097</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>68</v>
       </c>
       <c r="C69" t="n">
-        <v>0.746198</v>
+        <v>0.874981</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -2022,14 +2022,14 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>cand_0200</t>
+          <t>cand_0095</t>
         </is>
       </c>
       <c r="B70" t="n">
         <v>69</v>
       </c>
       <c r="C70" t="n">
-        <v>0.746146</v>
+        <v>0.87495</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -2045,14 +2045,14 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>cand_0182</t>
+          <t>cand_0684</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>70</v>
       </c>
       <c r="C71" t="n">
-        <v>0.745744</v>
+        <v>0.874335</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -2068,14 +2068,14 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>cand_0470</t>
+          <t>cand_0569</t>
         </is>
       </c>
       <c r="B72" t="n">
         <v>71</v>
       </c>
       <c r="C72" t="n">
-        <v>0.745729</v>
+        <v>0.874008</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -2091,14 +2091,14 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>cand_0837</t>
+          <t>cand_0140</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>72</v>
       </c>
       <c r="C73" t="n">
-        <v>0.7441489999999999</v>
+        <v>0.87243</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -2114,14 +2114,14 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>cand_0224</t>
+          <t>cand_0602</t>
         </is>
       </c>
       <c r="B74" t="n">
         <v>73</v>
       </c>
       <c r="C74" t="n">
-        <v>0.743936</v>
+        <v>0.872364</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -2137,14 +2137,14 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>cand_0203</t>
+          <t>cand_0182</t>
         </is>
       </c>
       <c r="B75" t="n">
         <v>74</v>
       </c>
       <c r="C75" t="n">
-        <v>0.743821</v>
+        <v>0.871928</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -2160,14 +2160,14 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>cand_0372</t>
+          <t>cand_0742</t>
         </is>
       </c>
       <c r="B76" t="n">
         <v>75</v>
       </c>
       <c r="C76" t="n">
-        <v>0.742072</v>
+        <v>0.871179</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -2183,14 +2183,14 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>cand_0160</t>
+          <t>cand_0487</t>
         </is>
       </c>
       <c r="B77" t="n">
         <v>76</v>
       </c>
       <c r="C77" t="n">
-        <v>0.740677</v>
+        <v>0.870816</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -2206,14 +2206,14 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>cand_0104</t>
+          <t>cand_0623</t>
         </is>
       </c>
       <c r="B78" t="n">
         <v>77</v>
       </c>
       <c r="C78" t="n">
-        <v>0.740398</v>
+        <v>0.869792</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -2236,7 +2236,7 @@
         <v>78</v>
       </c>
       <c r="C79" t="n">
-        <v>0.739785</v>
+        <v>0.869314</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -2252,14 +2252,14 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>cand_0193</t>
+          <t>cand_0106</t>
         </is>
       </c>
       <c r="B80" t="n">
         <v>79</v>
       </c>
       <c r="C80" t="n">
-        <v>0.739465</v>
+        <v>0.86837</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -2275,14 +2275,14 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>cand_0082</t>
+          <t>cand_0104</t>
         </is>
       </c>
       <c r="B81" t="n">
         <v>80</v>
       </c>
       <c r="C81" t="n">
-        <v>0.739363</v>
+        <v>0.8678</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -2298,14 +2298,14 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>cand_0090</t>
+          <t>cand_0200</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>81</v>
       </c>
       <c r="C82" t="n">
-        <v>0.738585</v>
+        <v>0.867635</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -2321,14 +2321,14 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>cand_0215</t>
+          <t>cand_0440</t>
         </is>
       </c>
       <c r="B83" t="n">
         <v>82</v>
       </c>
       <c r="C83" t="n">
-        <v>0.73754</v>
+        <v>0.867528</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -2344,14 +2344,14 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>cand_0001</t>
+          <t>cand_0220</t>
         </is>
       </c>
       <c r="B84" t="n">
         <v>83</v>
       </c>
       <c r="C84" t="n">
-        <v>0.7362300000000001</v>
+        <v>0.867247</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -2367,14 +2367,14 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>cand_0848</t>
+          <t>cand_0001</t>
         </is>
       </c>
       <c r="B85" t="n">
         <v>84</v>
       </c>
       <c r="C85" t="n">
-        <v>0.735649</v>
+        <v>0.865157</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -2390,14 +2390,14 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>cand_0095</t>
+          <t>cand_0224</t>
         </is>
       </c>
       <c r="B86" t="n">
         <v>85</v>
       </c>
       <c r="C86" t="n">
-        <v>0.734355</v>
+        <v>0.864165</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -2413,14 +2413,14 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>cand_0329</t>
+          <t>cand_0193</t>
         </is>
       </c>
       <c r="B87" t="n">
         <v>86</v>
       </c>
       <c r="C87" t="n">
-        <v>0.734247</v>
+        <v>0.862833</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -2436,14 +2436,14 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>cand_0487</t>
+          <t>cand_0739</t>
         </is>
       </c>
       <c r="B88" t="n">
         <v>87</v>
       </c>
       <c r="C88" t="n">
-        <v>0.7338170000000001</v>
+        <v>0.861432</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -2459,14 +2459,14 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>cand_0106</t>
+          <t>cand_0045</t>
         </is>
       </c>
       <c r="B89" t="n">
         <v>88</v>
       </c>
       <c r="C89" t="n">
-        <v>0.733656</v>
+        <v>0.859843</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -2482,14 +2482,14 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>cand_0742</t>
+          <t>cand_0329</t>
         </is>
       </c>
       <c r="B90" t="n">
         <v>89</v>
       </c>
       <c r="C90" t="n">
-        <v>0.733137</v>
+        <v>0.858787</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -2505,14 +2505,14 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>cand_0766</t>
+          <t>cand_0303</t>
         </is>
       </c>
       <c r="B91" t="n">
         <v>90</v>
       </c>
       <c r="C91" t="n">
-        <v>0.7324270000000001</v>
+        <v>0.857996</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -2528,14 +2528,14 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>cand_0205</t>
+          <t>cand_0926</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>91</v>
       </c>
       <c r="C92" t="n">
-        <v>0.731626</v>
+        <v>0.855799</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -2551,14 +2551,14 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>cand_0569</t>
+          <t>cand_0873</t>
         </is>
       </c>
       <c r="B93" t="n">
         <v>92</v>
       </c>
       <c r="C93" t="n">
-        <v>0.7316</v>
+        <v>0.855158</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -2574,14 +2574,14 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>cand_0276</t>
+          <t>cand_0496</t>
         </is>
       </c>
       <c r="B94" t="n">
         <v>93</v>
       </c>
       <c r="C94" t="n">
-        <v>0.729447</v>
+        <v>0.85221</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -2597,14 +2597,14 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>cand_0589</t>
+          <t>cand_0961</t>
         </is>
       </c>
       <c r="B95" t="n">
         <v>94</v>
       </c>
       <c r="C95" t="n">
-        <v>0.728411</v>
+        <v>0.851923</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -2620,14 +2620,14 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>cand_0620</t>
+          <t>cand_0180</t>
         </is>
       </c>
       <c r="B96" t="n">
         <v>95</v>
       </c>
       <c r="C96" t="n">
-        <v>0.726556</v>
+        <v>0.850419</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -2643,14 +2643,14 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>cand_0496</t>
+          <t>cand_0780</t>
         </is>
       </c>
       <c r="B97" t="n">
         <v>96</v>
       </c>
       <c r="C97" t="n">
-        <v>0.725615</v>
+        <v>0.84909</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -2666,14 +2666,14 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>cand_0071</t>
+          <t>cand_0624</t>
         </is>
       </c>
       <c r="B98" t="n">
         <v>97</v>
       </c>
       <c r="C98" t="n">
-        <v>0.724712</v>
+        <v>0.848418</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -2689,14 +2689,14 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>cand_0853</t>
+          <t>cand_0276</t>
         </is>
       </c>
       <c r="B99" t="n">
         <v>98</v>
       </c>
       <c r="C99" t="n">
-        <v>0.724674</v>
+        <v>0.846796</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -2712,14 +2712,14 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>cand_0456</t>
+          <t>cand_1000</t>
         </is>
       </c>
       <c r="B100" t="n">
         <v>99</v>
       </c>
       <c r="C100" t="n">
-        <v>0.723333</v>
+        <v>0.845328</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -2735,14 +2735,14 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>cand_0180</t>
+          <t>cand_0620</t>
         </is>
       </c>
       <c r="B101" t="n">
         <v>100</v>
       </c>
       <c r="C101" t="n">
-        <v>0.72283</v>
+        <v>0.843376</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix: resolve active job switching candidates queue refresh bug, frontend reload hydration, and technical council validation error
</commit_message>
<xml_diff>
--- a/data/submission.xlsx
+++ b/data/submission.xlsx
@@ -458,83 +458,83 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>cand_0593</t>
+          <t>cand_0841</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>0.961599</v>
+        <v>0.530625</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Strong Hire</t>
+          <t>Consider</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>cand_0936</t>
+          <t>cand_0491</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>0.946058</v>
+        <v>0.5168779999999999</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Strong Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>cand_0844</t>
+          <t>cand_0344</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>0.940347</v>
+        <v>0.490904</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Strong Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>cand_0419</t>
+          <t>cand_0805</t>
         </is>
       </c>
       <c r="B5" t="n">
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>0.938563</v>
+        <v>0.490758</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -543,136 +543,136 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Strong Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>cand_0156</t>
+          <t>cand_0197</t>
         </is>
       </c>
       <c r="B6" t="n">
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>0.938281</v>
+        <v>0.484422</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Strong Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>cand_0091</t>
+          <t>cand_0476</t>
         </is>
       </c>
       <c r="B7" t="n">
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>0.936964</v>
+        <v>0.48192</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Strong Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cand_0202</t>
+          <t>cand_0109</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>0.936826</v>
+        <v>0.480186</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Strong Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cand_0332</t>
+          <t>cand_0336</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>0.936738</v>
+        <v>0.478893</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Strong Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>cand_0737</t>
+          <t>cand_0776</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>0.933917</v>
+        <v>0.470161</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Strong Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>cand_0127</t>
+          <t>cand_0779</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>0.927675</v>
+        <v>0.467485</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -681,44 +681,44 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Strong Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>cand_0722</t>
+          <t>cand_0535</t>
         </is>
       </c>
       <c r="B12" t="n">
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>0.92675</v>
+        <v>0.46562</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Strong Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>cand_0062</t>
+          <t>cand_0725</t>
         </is>
       </c>
       <c r="B13" t="n">
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>0.926669</v>
+        <v>0.459415</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -727,67 +727,67 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Strong Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>cand_0592</t>
+          <t>cand_0544</t>
         </is>
       </c>
       <c r="B14" t="n">
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>0.9265679999999999</v>
+        <v>0.458621</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>cand_0402</t>
+          <t>cand_0291</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>0.924072</v>
+        <v>0.458114</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>cand_0621</t>
+          <t>cand_0206</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>0.923084</v>
+        <v>0.455468</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -796,21 +796,21 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>cand_0638</t>
+          <t>cand_0770</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" t="n">
-        <v>0.921457</v>
+        <v>0.453872</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -819,44 +819,44 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>cand_0337</t>
+          <t>cand_0298</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>0.918802</v>
+        <v>0.453042</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cand_0185</t>
+          <t>cand_0813</t>
         </is>
       </c>
       <c r="B19" t="n">
         <v>18</v>
       </c>
       <c r="C19" t="n">
-        <v>0.91777</v>
+        <v>0.45024</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -865,21 +865,21 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>cand_0088</t>
+          <t>cand_0521</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>19</v>
       </c>
       <c r="C20" t="n">
-        <v>0.915041</v>
+        <v>0.449267</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -888,21 +888,21 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>cand_0272</t>
+          <t>cand_0423</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>0.914465</v>
+        <v>0.449139</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -911,44 +911,44 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>cand_0956</t>
+          <t>cand_0114</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>21</v>
       </c>
       <c r="C22" t="n">
-        <v>0.9143559999999999</v>
+        <v>0.449104</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>cand_0170</t>
+          <t>cand_0085</t>
         </is>
       </c>
       <c r="B23" t="n">
         <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>0.912558</v>
+        <v>0.446946</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -957,21 +957,21 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>cand_0872</t>
+          <t>cand_0223</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>23</v>
       </c>
       <c r="C24" t="n">
-        <v>0.912301</v>
+        <v>0.446441</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -980,21 +980,21 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>cand_0462</t>
+          <t>cand_0120</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>24</v>
       </c>
       <c r="C25" t="n">
-        <v>0.911064</v>
+        <v>0.445551</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1003,44 +1003,44 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>cand_0886</t>
+          <t>cand_0700</t>
         </is>
       </c>
       <c r="B26" t="n">
         <v>25</v>
       </c>
       <c r="C26" t="n">
-        <v>0.909658</v>
+        <v>0.444617</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>cand_0111</t>
+          <t>cand_0292</t>
         </is>
       </c>
       <c r="B27" t="n">
         <v>26</v>
       </c>
       <c r="C27" t="n">
-        <v>0.909586</v>
+        <v>0.444159</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1049,21 +1049,21 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>cand_0647</t>
+          <t>cand_0727</t>
         </is>
       </c>
       <c r="B28" t="n">
         <v>27</v>
       </c>
       <c r="C28" t="n">
-        <v>0.9091</v>
+        <v>0.442539</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1072,21 +1072,21 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>cand_0269</t>
+          <t>cand_0585</t>
         </is>
       </c>
       <c r="B29" t="n">
         <v>28</v>
       </c>
       <c r="C29" t="n">
-        <v>0.908754</v>
+        <v>0.442351</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1095,67 +1095,67 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>cand_0494</t>
+          <t>cand_0164</t>
         </is>
       </c>
       <c r="B30" t="n">
         <v>29</v>
       </c>
       <c r="C30" t="n">
-        <v>0.908477</v>
+        <v>0.44056</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>cand_0826</t>
+          <t>cand_0925</t>
         </is>
       </c>
       <c r="B31" t="n">
         <v>30</v>
       </c>
       <c r="C31" t="n">
-        <v>0.906522</v>
+        <v>0.440294</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>cand_0021</t>
+          <t>cand_0755</t>
         </is>
       </c>
       <c r="B32" t="n">
         <v>31</v>
       </c>
       <c r="C32" t="n">
-        <v>0.906416</v>
+        <v>0.440136</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1164,113 +1164,113 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>cand_0246</t>
+          <t>cand_0626</t>
         </is>
       </c>
       <c r="B33" t="n">
         <v>32</v>
       </c>
       <c r="C33" t="n">
-        <v>0.905596</v>
+        <v>0.43955</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>cand_0505</t>
+          <t>cand_0549</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>33</v>
       </c>
       <c r="C34" t="n">
-        <v>0.904908</v>
+        <v>0.43894</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>cand_0902</t>
+          <t>cand_0558</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>34</v>
       </c>
       <c r="C35" t="n">
-        <v>0.903547</v>
+        <v>0.438517</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>cand_0529</t>
+          <t>cand_0799</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>35</v>
       </c>
       <c r="C36" t="n">
-        <v>0.902655</v>
+        <v>0.438295</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>cand_0122</t>
+          <t>cand_0510</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>36</v>
       </c>
       <c r="C37" t="n">
-        <v>0.90126</v>
+        <v>0.438237</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1279,44 +1279,44 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>cand_0809</t>
+          <t>cand_0528</t>
         </is>
       </c>
       <c r="B38" t="n">
         <v>37</v>
       </c>
       <c r="C38" t="n">
-        <v>0.899346</v>
+        <v>0.438012</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>cand_0281</t>
+          <t>cand_0948</t>
         </is>
       </c>
       <c r="B39" t="n">
         <v>38</v>
       </c>
       <c r="C39" t="n">
-        <v>0.898749</v>
+        <v>0.435755</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1325,21 +1325,21 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>cand_0508</t>
+          <t>cand_0668</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>39</v>
       </c>
       <c r="C40" t="n">
-        <v>0.898235</v>
+        <v>0.434522</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>cand_0501</t>
+          <t>cand_0736</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>40</v>
       </c>
       <c r="C41" t="n">
-        <v>0.8973</v>
+        <v>0.432527</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1371,21 +1371,21 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>cand_0618</t>
+          <t>cand_0050</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>41</v>
       </c>
       <c r="C42" t="n">
-        <v>0.897115</v>
+        <v>0.430881</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1394,21 +1394,21 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>cand_0998</t>
+          <t>cand_0993</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>42</v>
       </c>
       <c r="C43" t="n">
-        <v>0.8969200000000001</v>
+        <v>0.429001</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1417,67 +1417,67 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>cand_0335</t>
+          <t>cand_0395</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>43</v>
       </c>
       <c r="C44" t="n">
-        <v>0.896045</v>
+        <v>0.428341</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>cand_0856</t>
+          <t>cand_0964</t>
         </is>
       </c>
       <c r="B45" t="n">
         <v>44</v>
       </c>
       <c r="C45" t="n">
-        <v>0.895321</v>
+        <v>0.427881</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>cand_0427</t>
+          <t>cand_0334</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>45</v>
       </c>
       <c r="C46" t="n">
-        <v>0.894045</v>
+        <v>0.426307</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1486,44 +1486,44 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Hire</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>cand_0772</t>
+          <t>cand_0103</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>46</v>
       </c>
       <c r="C47" t="n">
-        <v>0.891879</v>
+        <v>0.4262</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>cand_0203</t>
+          <t>cand_0619</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>47</v>
       </c>
       <c r="C48" t="n">
-        <v>0.890361</v>
+        <v>0.425083</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1532,21 +1532,21 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>cand_0221</t>
+          <t>cand_0105</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>48</v>
       </c>
       <c r="C49" t="n">
-        <v>0.889374</v>
+        <v>0.423567</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
@@ -1555,21 +1555,21 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>cand_0831</t>
+          <t>cand_0319</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>49</v>
       </c>
       <c r="C50" t="n">
-        <v>0.888646</v>
+        <v>0.42293</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -1578,21 +1578,21 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>cand_0079</t>
+          <t>cand_0649</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>50</v>
       </c>
       <c r="C51" t="n">
-        <v>0.888616</v>
+        <v>0.422031</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -1601,67 +1601,67 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>cand_0470</t>
+          <t>cand_0705</t>
         </is>
       </c>
       <c r="B52" t="n">
         <v>51</v>
       </c>
       <c r="C52" t="n">
-        <v>0.888313</v>
+        <v>0.421436</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>cand_0163</t>
+          <t>cand_0230</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>52</v>
       </c>
       <c r="C53" t="n">
-        <v>0.886999</v>
+        <v>0.420482</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>cand_0433</t>
+          <t>cand_0782</t>
         </is>
       </c>
       <c r="B54" t="n">
         <v>53</v>
       </c>
       <c r="C54" t="n">
-        <v>0.886518</v>
+        <v>0.419321</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
@@ -1670,67 +1670,67 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>cand_0372</t>
+          <t>cand_0175</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>54</v>
       </c>
       <c r="C55" t="n">
-        <v>0.885612</v>
+        <v>0.419119</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>cand_0063</t>
+          <t>cand_0662</t>
         </is>
       </c>
       <c r="B56" t="n">
         <v>55</v>
       </c>
       <c r="C56" t="n">
-        <v>0.885588</v>
+        <v>0.419018</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>cand_0773</t>
+          <t>cand_0650</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>56</v>
       </c>
       <c r="C57" t="n">
-        <v>0.885136</v>
+        <v>0.417528</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
@@ -1739,21 +1739,21 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>cand_0837</t>
+          <t>cand_0749</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>57</v>
       </c>
       <c r="C58" t="n">
-        <v>0.884973</v>
+        <v>0.416076</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
@@ -1762,182 +1762,182 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>cand_0653</t>
+          <t>cand_0570</t>
         </is>
       </c>
       <c r="B59" t="n">
         <v>58</v>
       </c>
       <c r="C59" t="n">
-        <v>0.882467</v>
+        <v>0.415301</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>cand_0965</t>
+          <t>cand_0420</t>
         </is>
       </c>
       <c r="B60" t="n">
         <v>59</v>
       </c>
       <c r="C60" t="n">
-        <v>0.882307</v>
+        <v>0.415183</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>cand_0483</t>
+          <t>cand_0388</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>60</v>
       </c>
       <c r="C61" t="n">
-        <v>0.881575</v>
+        <v>0.414901</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>cand_0090</t>
+          <t>cand_0008</t>
         </is>
       </c>
       <c r="B62" t="n">
         <v>61</v>
       </c>
       <c r="C62" t="n">
-        <v>0.881121</v>
+        <v>0.413732</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>cand_0363</t>
+          <t>cand_0581</t>
         </is>
       </c>
       <c r="B63" t="n">
         <v>62</v>
       </c>
       <c r="C63" t="n">
-        <v>0.8806890000000001</v>
+        <v>0.412862</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>cand_0253</t>
+          <t>cand_0010</t>
         </is>
       </c>
       <c r="B64" t="n">
         <v>63</v>
       </c>
       <c r="C64" t="n">
-        <v>0.878386</v>
+        <v>0.410565</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>cand_0766</t>
+          <t>cand_0763</t>
         </is>
       </c>
       <c r="B65" t="n">
         <v>64</v>
       </c>
       <c r="C65" t="n">
-        <v>0.878365</v>
+        <v>0.410508</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>cand_0160</t>
+          <t>cand_0671</t>
         </is>
       </c>
       <c r="B66" t="n">
         <v>65</v>
       </c>
       <c r="C66" t="n">
-        <v>0.878045</v>
+        <v>0.40957</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -1946,44 +1946,44 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>cand_0082</t>
+          <t>cand_0740</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>66</v>
       </c>
       <c r="C67" t="n">
-        <v>0.876559</v>
+        <v>0.40908</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>cand_0588</t>
+          <t>cand_0927</t>
         </is>
       </c>
       <c r="B68" t="n">
         <v>67</v>
       </c>
       <c r="C68" t="n">
-        <v>0.875894</v>
+        <v>0.408229</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -1992,67 +1992,67 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>cand_0097</t>
+          <t>cand_0489</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>68</v>
       </c>
       <c r="C69" t="n">
-        <v>0.874981</v>
+        <v>0.407932</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>cand_0095</t>
+          <t>cand_0119</t>
         </is>
       </c>
       <c r="B70" t="n">
         <v>69</v>
       </c>
       <c r="C70" t="n">
-        <v>0.87495</v>
+        <v>0.407902</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>cand_0684</t>
+          <t>cand_0610</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>70</v>
       </c>
       <c r="C71" t="n">
-        <v>0.874335</v>
+        <v>0.407306</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -2061,90 +2061,90 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>cand_0569</t>
+          <t>cand_0966</t>
         </is>
       </c>
       <c r="B72" t="n">
         <v>71</v>
       </c>
       <c r="C72" t="n">
-        <v>0.874008</v>
+        <v>0.406302</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>cand_0140</t>
+          <t>cand_0480</t>
         </is>
       </c>
       <c r="B73" t="n">
         <v>72</v>
       </c>
       <c r="C73" t="n">
-        <v>0.87243</v>
+        <v>0.404414</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>cand_0602</t>
+          <t>cand_0430</t>
         </is>
       </c>
       <c r="B74" t="n">
         <v>73</v>
       </c>
       <c r="C74" t="n">
-        <v>0.872364</v>
+        <v>0.40372</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>cand_0182</t>
+          <t>cand_0655</t>
         </is>
       </c>
       <c r="B75" t="n">
         <v>74</v>
       </c>
       <c r="C75" t="n">
-        <v>0.871928</v>
+        <v>0.403489</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -2153,21 +2153,21 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>cand_0742</t>
+          <t>cand_0417</t>
         </is>
       </c>
       <c r="B76" t="n">
         <v>75</v>
       </c>
       <c r="C76" t="n">
-        <v>0.871179</v>
+        <v>0.4033</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -2176,25 +2176,25 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Consider</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>cand_0487</t>
+          <t>cand_0214</t>
         </is>
       </c>
       <c r="B77" t="n">
         <v>76</v>
       </c>
       <c r="C77" t="n">
-        <v>0.870816</v>
+        <v>0.403212</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -2206,18 +2206,18 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>cand_0623</t>
+          <t>cand_0633</t>
         </is>
       </c>
       <c r="B78" t="n">
         <v>77</v>
       </c>
       <c r="C78" t="n">
-        <v>0.869792</v>
+        <v>0.401445</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -2229,18 +2229,18 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>cand_0644</t>
+          <t>cand_0879</t>
         </is>
       </c>
       <c r="B79" t="n">
         <v>78</v>
       </c>
       <c r="C79" t="n">
-        <v>0.869314</v>
+        <v>0.401076</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -2252,18 +2252,18 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>cand_0106</t>
+          <t>cand_0784</t>
         </is>
       </c>
       <c r="B80" t="n">
         <v>79</v>
       </c>
       <c r="C80" t="n">
-        <v>0.86837</v>
+        <v>0.401013</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -2275,18 +2275,18 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>cand_0104</t>
+          <t>cand_0449</t>
         </is>
       </c>
       <c r="B81" t="n">
         <v>80</v>
       </c>
       <c r="C81" t="n">
-        <v>0.8678</v>
+        <v>0.398762</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -2298,14 +2298,14 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>cand_0200</t>
+          <t>cand_0448</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>81</v>
       </c>
       <c r="C82" t="n">
-        <v>0.867635</v>
+        <v>0.396985</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -2321,18 +2321,18 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>cand_0440</t>
+          <t>cand_0604</t>
         </is>
       </c>
       <c r="B83" t="n">
         <v>82</v>
       </c>
       <c r="C83" t="n">
-        <v>0.867528</v>
+        <v>0.396557</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -2344,18 +2344,18 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>cand_0220</t>
+          <t>cand_0760</t>
         </is>
       </c>
       <c r="B84" t="n">
         <v>83</v>
       </c>
       <c r="C84" t="n">
-        <v>0.867247</v>
+        <v>0.395771</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -2367,14 +2367,14 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>cand_0001</t>
+          <t>cand_0616</t>
         </is>
       </c>
       <c r="B85" t="n">
         <v>84</v>
       </c>
       <c r="C85" t="n">
-        <v>0.865157</v>
+        <v>0.393412</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -2390,14 +2390,14 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>cand_0224</t>
+          <t>cand_0797</t>
         </is>
       </c>
       <c r="B86" t="n">
         <v>85</v>
       </c>
       <c r="C86" t="n">
-        <v>0.864165</v>
+        <v>0.3919</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -2413,14 +2413,14 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>cand_0193</t>
+          <t>cand_0032</t>
         </is>
       </c>
       <c r="B87" t="n">
         <v>86</v>
       </c>
       <c r="C87" t="n">
-        <v>0.862833</v>
+        <v>0.391483</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -2436,14 +2436,14 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>cand_0739</t>
+          <t>cand_0142</t>
         </is>
       </c>
       <c r="B88" t="n">
         <v>87</v>
       </c>
       <c r="C88" t="n">
-        <v>0.861432</v>
+        <v>0.387665</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -2459,14 +2459,14 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>cand_0045</t>
+          <t>cand_0447</t>
         </is>
       </c>
       <c r="B89" t="n">
         <v>88</v>
       </c>
       <c r="C89" t="n">
-        <v>0.859843</v>
+        <v>0.386949</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -2482,18 +2482,18 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>cand_0329</t>
+          <t>cand_0656</t>
         </is>
       </c>
       <c r="B90" t="n">
         <v>89</v>
       </c>
       <c r="C90" t="n">
-        <v>0.858787</v>
+        <v>0.386527</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -2505,14 +2505,14 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>cand_0303</t>
+          <t>cand_0913</t>
         </is>
       </c>
       <c r="B91" t="n">
         <v>90</v>
       </c>
       <c r="C91" t="n">
-        <v>0.857996</v>
+        <v>0.384771</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -2528,18 +2528,18 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>cand_0926</t>
+          <t>cand_0118</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>91</v>
       </c>
       <c r="C92" t="n">
-        <v>0.855799</v>
+        <v>0.38417</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
@@ -2551,14 +2551,14 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>cand_0873</t>
+          <t>cand_0207</t>
         </is>
       </c>
       <c r="B93" t="n">
         <v>92</v>
       </c>
       <c r="C93" t="n">
-        <v>0.855158</v>
+        <v>0.377373</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -2567,21 +2567,21 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Reject</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>cand_0496</t>
+          <t>cand_0138</t>
         </is>
       </c>
       <c r="B94" t="n">
         <v>93</v>
       </c>
       <c r="C94" t="n">
-        <v>0.85221</v>
+        <v>0.377332</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -2590,21 +2590,21 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Reject</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>cand_0961</t>
+          <t>cand_0157</t>
         </is>
       </c>
       <c r="B95" t="n">
         <v>94</v>
       </c>
       <c r="C95" t="n">
-        <v>0.851923</v>
+        <v>0.374804</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -2613,21 +2613,21 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Reject</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>cand_0180</t>
+          <t>cand_0023</t>
         </is>
       </c>
       <c r="B96" t="n">
         <v>95</v>
       </c>
       <c r="C96" t="n">
-        <v>0.850419</v>
+        <v>0.373587</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -2636,21 +2636,21 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Reject</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>cand_0780</t>
+          <t>cand_0218</t>
         </is>
       </c>
       <c r="B97" t="n">
         <v>96</v>
       </c>
       <c r="C97" t="n">
-        <v>0.84909</v>
+        <v>0.370664</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -2659,21 +2659,21 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Reject</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>cand_0624</t>
+          <t>cand_0411</t>
         </is>
       </c>
       <c r="B98" t="n">
         <v>97</v>
       </c>
       <c r="C98" t="n">
-        <v>0.848418</v>
+        <v>0.36608</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -2682,21 +2682,21 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Reject</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>cand_0276</t>
+          <t>cand_0064</t>
         </is>
       </c>
       <c r="B99" t="n">
         <v>98</v>
       </c>
       <c r="C99" t="n">
-        <v>0.846796</v>
+        <v>0.362906</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -2705,44 +2705,44 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Reject</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>cand_1000</t>
+          <t>cand_0060</t>
         </is>
       </c>
       <c r="B100" t="n">
         <v>99</v>
       </c>
       <c r="C100" t="n">
-        <v>0.845328</v>
+        <v>0.361967</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Reject</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>cand_0620</t>
+          <t>cand_0815</t>
         </is>
       </c>
       <c r="B101" t="n">
         <v>100</v>
       </c>
       <c r="C101" t="n">
-        <v>0.843376</v>
+        <v>0.356535</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Reject</t>
         </is>
       </c>
     </row>

</xml_diff>